<commit_message>
refactor(blue): consolida regras de gamificacao
</commit_message>
<xml_diff>
--- a/docs/ATDD-Case-AC1.xlsx
+++ b/docs/ATDD-Case-AC1.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\edubn\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\edubn\OneDrive\Documentos\Nova pasta\gamificacao-educacao-continuada\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E97C68A-4131-4C75-8A1F-D5E8E5EF4ED8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A2C14E9-E61D-4B0E-922A-553B960E6ED9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="pb" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="72">
   <si>
     <t>PRODUCT BACKLOG</t>
   </si>
@@ -278,9 +278,6 @@
     </r>
   </si>
   <si>
-    <t>ALUNO</t>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">Como </t>
     </r>
@@ -445,6 +442,15 @@
   </si>
   <si>
     <t>João Victor Cardoso Engler Rizzi de Araujo</t>
+  </si>
+  <si>
+    <t>Eduardo</t>
+  </si>
+  <si>
+    <t>Khevyn</t>
+  </si>
+  <si>
+    <t>João</t>
   </si>
 </sst>
 </file>
@@ -1177,10 +1183,10 @@
         <v>1</v>
       </c>
       <c r="B5" s="23" t="s">
+        <v>69</v>
+      </c>
+      <c r="C5" s="21" t="s">
         <v>38</v>
-      </c>
-      <c r="C5" s="21" t="s">
-        <v>39</v>
       </c>
       <c r="D5" s="22" t="s">
         <v>36</v>
@@ -1190,30 +1196,30 @@
       </c>
       <c r="F5" s="39"/>
       <c r="G5" s="21" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="H5" s="21" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="I5" s="21" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="J5" s="7"/>
       <c r="K5" s="21" t="s">
+        <v>44</v>
+      </c>
+      <c r="L5" s="21" t="s">
         <v>45</v>
-      </c>
-      <c r="L5" s="21" t="s">
-        <v>46</v>
       </c>
       <c r="M5" s="39"/>
       <c r="N5" s="24" t="s">
+        <v>47</v>
+      </c>
+      <c r="O5" s="24" t="s">
         <v>48</v>
       </c>
-      <c r="O5" s="24" t="s">
+      <c r="P5" s="26" t="s">
         <v>49</v>
-      </c>
-      <c r="P5" s="26" t="s">
-        <v>50</v>
       </c>
       <c r="Q5" s="27"/>
       <c r="R5" s="27"/>
@@ -1224,43 +1230,43 @@
         <v>2</v>
       </c>
       <c r="B6" s="23" t="s">
+        <v>70</v>
+      </c>
+      <c r="C6" s="21" t="s">
         <v>38</v>
       </c>
-      <c r="C6" s="21" t="s">
+      <c r="D6" s="22" t="s">
         <v>39</v>
       </c>
-      <c r="D6" s="22" t="s">
+      <c r="E6" s="22" t="s">
         <v>40</v>
-      </c>
-      <c r="E6" s="22" t="s">
-        <v>41</v>
       </c>
       <c r="F6" s="39"/>
       <c r="G6" s="21" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="H6" s="21" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="I6" s="21" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="J6" s="6"/>
       <c r="K6" s="6" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="L6" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="M6" s="39"/>
       <c r="N6" s="21" t="s">
+        <v>53</v>
+      </c>
+      <c r="O6" s="21" t="s">
         <v>54</v>
       </c>
-      <c r="O6" s="21" t="s">
+      <c r="P6" s="26" t="s">
         <v>55</v>
-      </c>
-      <c r="P6" s="26" t="s">
-        <v>56</v>
       </c>
       <c r="Q6" s="27"/>
       <c r="R6" s="27"/>
@@ -1271,43 +1277,43 @@
         <v>3</v>
       </c>
       <c r="B7" s="23" t="s">
+        <v>71</v>
+      </c>
+      <c r="C7" s="21" t="s">
         <v>38</v>
       </c>
-      <c r="C7" s="21" t="s">
-        <v>39</v>
-      </c>
       <c r="D7" s="22" t="s">
+        <v>41</v>
+      </c>
+      <c r="E7" s="22" t="s">
         <v>42</v>
-      </c>
-      <c r="E7" s="22" t="s">
-        <v>43</v>
       </c>
       <c r="F7" s="39"/>
       <c r="G7" s="21" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="H7" s="21" t="s">
+        <v>56</v>
+      </c>
+      <c r="I7" s="21" t="s">
         <v>57</v>
-      </c>
-      <c r="I7" s="21" t="s">
-        <v>58</v>
       </c>
       <c r="J7" s="6"/>
       <c r="K7" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="L7" s="25" t="s">
         <v>59</v>
-      </c>
-      <c r="L7" s="25" t="s">
-        <v>60</v>
       </c>
       <c r="M7" s="39"/>
       <c r="N7" s="21" t="s">
+        <v>60</v>
+      </c>
+      <c r="O7" s="21" t="s">
         <v>61</v>
       </c>
-      <c r="O7" s="21" t="s">
+      <c r="P7" s="26" t="s">
         <v>62</v>
-      </c>
-      <c r="P7" s="26" t="s">
-        <v>63</v>
       </c>
       <c r="Q7" s="27"/>
       <c r="R7" s="27"/>
@@ -2391,15 +2397,15 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B1" t="s">
         <v>66</v>
-      </c>
-      <c r="B1" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B2">
         <v>211466</v>
@@ -2407,7 +2413,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B3">
         <v>223761</v>
@@ -2415,7 +2421,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B4">
         <v>236602</v>

</xml_diff>